<commit_message>
DASS-21/42: add likert anchors for 10 langs; fix license metadata
Add missing likert_1–4 anchor labels and question_head for bg, hi, ja,
ko, mn, ne, ru, sl, th, zh in DASS21.osd (all 10) and DASS42.osd (7;
mn/ne/ru not present in DASS42). Text extracted from official UNSW PDFs
downloaded to misc/DASS/.

Fix license fields on both scales: was "Public Domain" with no evidence;
now documented with license_explanation quoting the UNSW DASS FAQ ("The
DASS questionnaire is public domain, and so permission is not needed to
use it") and license_url pointing to the FAQ anchor. Add DASS-21 and
DASS-42 rows to permissions/permissions.xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/permissions/permissions.xlsx
+++ b/permissions/permissions.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="97">
   <si>
     <t xml:space="preserve">This identfiies scales for which we maintain documentation of permissions, either granted to OpenScales directly or documented publicly elsewhere.</t>
   </si>
@@ -281,6 +281,36 @@
   </si>
   <si>
     <t xml:space="preserve">openscales/BSS-PB.osd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DASS-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depression Anxiety Stress Scales 21-item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">openscales/DASS21/DASS21.osd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www2.psy.unsw.edu.au/groups/dass/DASSFAQ.htm#_3.__How_do_I_get_permission_to_use_</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNSW (Lovibond &amp; Lovibond)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public Domain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DASS-42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depression Anxiety Stress Scales 42-item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">openscales/DASS42/DASS42.osd</t>
   </si>
 </sst>
 </file>
@@ -498,12 +528,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="21.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="64.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="64.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.61"/>
@@ -947,7 +977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>66</v>
       </c>
@@ -970,7 +1000,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>69</v>
       </c>
@@ -993,7 +1023,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>72</v>
       </c>
@@ -1016,7 +1046,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>75</v>
       </c>
@@ -1039,7 +1069,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>78</v>
       </c>
@@ -1062,7 +1092,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>81</v>
       </c>
@@ -1085,7 +1115,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>84</v>
       </c>
@@ -1106,6 +1136,52 @@
       </c>
       <c r="G29" s="1" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>